<commit_message>
fix tokz. inner signals from MTZ deleted (pusk st)
</commit_message>
<xml_diff>
--- a/mode_docx_gen/pmi_tokz/lzt_modes/ЛЗТ_4.xlsx
+++ b/mode_docx_gen/pmi_tokz/lzt_modes/ЛЗТ_4.xlsx
@@ -587,8 +587,8 @@
       <c r="J2" t="n">
         <v>0</v>
       </c>
-      <c r="K2" t="n">
-        <v>0</v>
+      <c r="K2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="L2" s="2" t="n">
         <v>1</v>
@@ -894,8 +894,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>0</v>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
@@ -933,26 +933,26 @@
       <c r="M2" t="n">
         <v>0</v>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -1392,16 +1392,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="Z2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1412,16 +1412,16 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AB2" s="2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AC2" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="AD2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1432,29 +1432,29 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AF2" s="2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG2" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="AH2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AI2" s="2" t="inlineStr">
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ2" s="2" t="inlineStr">
         <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>0</t>
         </is>
       </c>
       <c r="AK2" t="inlineStr">

</xml_diff>